<commit_message>
Add deliverable phase ordering for project scenarios
Implements helper functions to rank and sort deliverables based on phase and custom overrides, and integrates this sorting logic into the API build process before scenario assignment.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 4c2d841a-8e9c-42d2-a44f-f90dc1c78202
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/0e11dc90-618e-44e7-83a8-20eddbc22afb/4c2d841a-8e9c-42d2-a44f-f90dc1c78202/cqhrmiR
</commit_message>
<xml_diff>
--- a/RFP_Brief_ First on SoundCloud 2021 Campaign - Scenario A - Workfront Export.xlsx
+++ b/RFP_Brief_ First on SoundCloud 2021 Campaign - Scenario A - Workfront Export.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q112"/>
+  <dimension ref="A1:R112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -508,10 +508,15 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>Service_Department</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>Rate_USD</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Price_USD</t>
         </is>
@@ -553,10 +558,11 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" s="3" t="n">
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="Q2" s="2" t="n">
+      <c r="R2" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -606,10 +612,11 @@
           <t>Core/T2_MediumVolume</t>
         </is>
       </c>
-      <c r="P3" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q3" s="2" t="n">
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R3" s="2" t="n">
         <v>44265</v>
       </c>
     </row>
@@ -663,10 +670,11 @@
       </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
-      <c r="P4" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q4" s="2" t="n">
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R4" s="2" t="n">
         <v>9750</v>
       </c>
     </row>
@@ -732,10 +740,11 @@
       </c>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
-      <c r="P5" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q5" s="2" t="n">
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R5" s="2" t="n">
         <v>390</v>
       </c>
     </row>
@@ -801,10 +810,11 @@
       </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
-      <c r="P6" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q6" s="2" t="n">
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R6" s="2" t="n">
         <v>780</v>
       </c>
     </row>
@@ -870,10 +880,11 @@
       </c>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
-      <c r="P7" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q7" s="2" t="n">
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R7" s="2" t="n">
         <v>8580</v>
       </c>
     </row>
@@ -927,10 +938,11 @@
       </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q8" s="2" t="n">
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R8" s="2" t="n">
         <v>3315</v>
       </c>
     </row>
@@ -996,10 +1008,11 @@
       </c>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
-      <c r="P9" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q9" s="2" t="n">
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R9" s="2" t="n">
         <v>3315</v>
       </c>
     </row>
@@ -1053,10 +1066,11 @@
       </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q10" s="2" t="n">
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R10" s="2" t="n">
         <v>3315</v>
       </c>
     </row>
@@ -1122,10 +1136,11 @@
       </c>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
-      <c r="P11" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q11" s="2" t="n">
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R11" s="2" t="n">
         <v>3315</v>
       </c>
     </row>
@@ -1179,10 +1194,11 @@
       </c>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
-      <c r="P12" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q12" s="2" t="n">
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R12" s="2" t="n">
         <v>8385</v>
       </c>
     </row>
@@ -1248,10 +1264,11 @@
       </c>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
-      <c r="P13" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q13" s="2" t="n">
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R13" s="2" t="n">
         <v>585</v>
       </c>
     </row>
@@ -1317,10 +1334,11 @@
       </c>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
-      <c r="P14" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q14" s="2" t="n">
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R14" s="2" t="n">
         <v>1170</v>
       </c>
     </row>
@@ -1386,10 +1404,11 @@
       </c>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
-      <c r="P15" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q15" s="2" t="n">
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R15" s="2" t="n">
         <v>6630</v>
       </c>
     </row>
@@ -1443,10 +1462,11 @@
       </c>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
-      <c r="P16" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q16" s="2" t="n">
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R16" s="2" t="n">
         <v>8385</v>
       </c>
     </row>
@@ -1512,10 +1532,11 @@
       </c>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
-      <c r="P17" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q17" s="2" t="n">
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R17" s="2" t="n">
         <v>585</v>
       </c>
     </row>
@@ -1581,10 +1602,11 @@
       </c>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q18" s="2" t="n">
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R18" s="2" t="n">
         <v>1170</v>
       </c>
     </row>
@@ -1650,10 +1672,11 @@
       </c>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
-      <c r="P19" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q19" s="2" t="n">
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R19" s="2" t="n">
         <v>6630</v>
       </c>
     </row>
@@ -1707,10 +1730,11 @@
       </c>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
-      <c r="P20" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q20" s="2" t="n">
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R20" s="2" t="n">
         <v>1365</v>
       </c>
     </row>
@@ -1776,10 +1800,11 @@
       </c>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
-      <c r="P21" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q21" s="2" t="n">
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R21" s="2" t="n">
         <v>585</v>
       </c>
     </row>
@@ -1845,10 +1870,11 @@
       </c>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
-      <c r="P22" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q22" s="2" t="n">
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R22" s="2" t="n">
         <v>780</v>
       </c>
     </row>
@@ -1902,10 +1928,11 @@
       </c>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
-      <c r="P23" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q23" s="2" t="n">
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R23" s="2" t="n">
         <v>1365</v>
       </c>
     </row>
@@ -1971,10 +1998,11 @@
       </c>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
-      <c r="P24" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q24" s="2" t="n">
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R24" s="2" t="n">
         <v>585</v>
       </c>
     </row>
@@ -2040,10 +2068,11 @@
       </c>
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
-      <c r="P25" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q25" s="2" t="n">
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R25" s="2" t="n">
         <v>780</v>
       </c>
     </row>
@@ -2097,10 +2126,11 @@
       </c>
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
-      <c r="P26" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q26" s="2" t="n">
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R26" s="2" t="n">
         <v>975</v>
       </c>
     </row>
@@ -2166,10 +2196,11 @@
       </c>
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
-      <c r="P27" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q27" s="2" t="n">
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R27" s="2" t="n">
         <v>585</v>
       </c>
     </row>
@@ -2235,10 +2266,11 @@
       </c>
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
-      <c r="P28" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q28" s="2" t="n">
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R28" s="2" t="n">
         <v>390</v>
       </c>
     </row>
@@ -2292,10 +2324,11 @@
       </c>
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
-      <c r="P29" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q29" s="2" t="n">
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R29" s="2" t="n">
         <v>1365</v>
       </c>
     </row>
@@ -2361,10 +2394,11 @@
       </c>
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
-      <c r="P30" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q30" s="2" t="n">
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R30" s="2" t="n">
         <v>585</v>
       </c>
     </row>
@@ -2430,10 +2464,11 @@
       </c>
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
-      <c r="P31" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q31" s="2" t="n">
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R31" s="2" t="n">
         <v>780</v>
       </c>
     </row>
@@ -2487,10 +2522,11 @@
       </c>
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
-      <c r="P32" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q32" s="2" t="n">
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R32" s="2" t="n">
         <v>1365</v>
       </c>
     </row>
@@ -2556,10 +2592,11 @@
       </c>
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr"/>
-      <c r="P33" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q33" s="2" t="n">
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R33" s="2" t="n">
         <v>585</v>
       </c>
     </row>
@@ -2625,10 +2662,11 @@
       </c>
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr"/>
-      <c r="P34" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q34" s="2" t="n">
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R34" s="2" t="n">
         <v>780</v>
       </c>
     </row>
@@ -2682,10 +2720,11 @@
       </c>
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
-      <c r="P35" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q35" s="2" t="n">
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R35" s="2" t="n">
         <v>975</v>
       </c>
     </row>
@@ -2751,10 +2790,11 @@
       </c>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
-      <c r="P36" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q36" s="2" t="n">
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R36" s="2" t="n">
         <v>585</v>
       </c>
     </row>
@@ -2820,10 +2860,11 @@
       </c>
       <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr"/>
-      <c r="P37" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q37" s="2" t="n">
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R37" s="2" t="n">
         <v>390</v>
       </c>
     </row>
@@ -2877,10 +2918,11 @@
       </c>
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
-      <c r="P38" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q38" s="2" t="n">
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R38" s="2" t="n">
         <v>780</v>
       </c>
     </row>
@@ -2946,10 +2988,11 @@
       </c>
       <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr"/>
-      <c r="P39" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q39" s="2" t="n">
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R39" s="2" t="n">
         <v>780</v>
       </c>
     </row>
@@ -3003,10 +3046,11 @@
       </c>
       <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr"/>
-      <c r="P40" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q40" s="2" t="n">
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R40" s="2" t="n">
         <v>780</v>
       </c>
     </row>
@@ -3072,10 +3116,11 @@
       </c>
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
-      <c r="P41" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q41" s="2" t="n">
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R41" s="2" t="n">
         <v>390</v>
       </c>
     </row>
@@ -3141,10 +3186,11 @@
       </c>
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
-      <c r="P42" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q42" s="2" t="n">
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R42" s="2" t="n">
         <v>390</v>
       </c>
     </row>
@@ -3198,10 +3244,11 @@
       </c>
       <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
-      <c r="P43" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q43" s="2" t="n">
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R43" s="2" t="n">
         <v>780</v>
       </c>
     </row>
@@ -3267,10 +3314,11 @@
       </c>
       <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr"/>
-      <c r="P44" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q44" s="2" t="n">
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R44" s="2" t="n">
         <v>390</v>
       </c>
     </row>
@@ -3336,10 +3384,11 @@
       </c>
       <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
-      <c r="P45" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q45" s="2" t="n">
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R45" s="2" t="n">
         <v>390</v>
       </c>
     </row>
@@ -3393,10 +3442,11 @@
       </c>
       <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr"/>
-      <c r="P46" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q46" s="2" t="n">
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R46" s="2" t="n">
         <v>1365</v>
       </c>
     </row>
@@ -3462,10 +3512,11 @@
       </c>
       <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr"/>
-      <c r="P47" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q47" s="2" t="n">
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R47" s="2" t="n">
         <v>585</v>
       </c>
     </row>
@@ -3531,10 +3582,11 @@
       </c>
       <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr"/>
-      <c r="P48" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q48" s="2" t="n">
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R48" s="2" t="n">
         <v>780</v>
       </c>
     </row>
@@ -3588,10 +3640,11 @@
           <t>Core/T2_MediumVolume</t>
         </is>
       </c>
-      <c r="P49" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q49" s="2" t="n">
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R49" s="2" t="n">
         <v>36660</v>
       </c>
     </row>
@@ -3645,10 +3698,11 @@
       </c>
       <c r="N50" t="inlineStr"/>
       <c r="O50" t="inlineStr"/>
-      <c r="P50" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q50" s="2" t="n">
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R50" s="2" t="n">
         <v>390</v>
       </c>
     </row>
@@ -3714,10 +3768,11 @@
       </c>
       <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr"/>
-      <c r="P51" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q51" s="2" t="n">
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R51" s="2" t="n">
         <v>195</v>
       </c>
     </row>
@@ -3783,10 +3838,11 @@
       </c>
       <c r="N52" t="inlineStr"/>
       <c r="O52" t="inlineStr"/>
-      <c r="P52" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q52" s="2" t="n">
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R52" s="2" t="n">
         <v>195</v>
       </c>
     </row>
@@ -3840,10 +3896,11 @@
       </c>
       <c r="N53" t="inlineStr"/>
       <c r="O53" t="inlineStr"/>
-      <c r="P53" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q53" s="2" t="n">
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R53" s="2" t="n">
         <v>975</v>
       </c>
     </row>
@@ -3909,10 +3966,11 @@
       </c>
       <c r="N54" t="inlineStr"/>
       <c r="O54" t="inlineStr"/>
-      <c r="P54" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q54" s="2" t="n">
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R54" s="2" t="n">
         <v>195</v>
       </c>
     </row>
@@ -3978,10 +4036,11 @@
       </c>
       <c r="N55" t="inlineStr"/>
       <c r="O55" t="inlineStr"/>
-      <c r="P55" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q55" s="2" t="n">
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R55" s="2" t="n">
         <v>780</v>
       </c>
     </row>
@@ -4035,10 +4094,11 @@
       </c>
       <c r="N56" t="inlineStr"/>
       <c r="O56" t="inlineStr"/>
-      <c r="P56" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q56" s="2" t="n">
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R56" s="2" t="n">
         <v>3315</v>
       </c>
     </row>
@@ -4104,10 +4164,11 @@
       </c>
       <c r="N57" t="inlineStr"/>
       <c r="O57" t="inlineStr"/>
-      <c r="P57" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q57" s="2" t="n">
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R57" s="2" t="n">
         <v>3315</v>
       </c>
     </row>
@@ -4161,10 +4222,11 @@
       </c>
       <c r="N58" t="inlineStr"/>
       <c r="O58" t="inlineStr"/>
-      <c r="P58" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q58" s="2" t="n">
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R58" s="2" t="n">
         <v>4875</v>
       </c>
     </row>
@@ -4230,10 +4292,11 @@
       </c>
       <c r="N59" t="inlineStr"/>
       <c r="O59" t="inlineStr"/>
-      <c r="P59" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q59" s="2" t="n">
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R59" s="2" t="n">
         <v>4875</v>
       </c>
     </row>
@@ -4287,10 +4350,11 @@
       </c>
       <c r="N60" t="inlineStr"/>
       <c r="O60" t="inlineStr"/>
-      <c r="P60" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q60" s="2" t="n">
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R60" s="2" t="n">
         <v>3315</v>
       </c>
     </row>
@@ -4356,10 +4420,11 @@
       </c>
       <c r="N61" t="inlineStr"/>
       <c r="O61" t="inlineStr"/>
-      <c r="P61" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q61" s="2" t="n">
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R61" s="2" t="n">
         <v>1755</v>
       </c>
     </row>
@@ -4425,10 +4490,11 @@
       </c>
       <c r="N62" t="inlineStr"/>
       <c r="O62" t="inlineStr"/>
-      <c r="P62" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q62" s="2" t="n">
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R62" s="2" t="n">
         <v>390</v>
       </c>
     </row>
@@ -4494,10 +4560,11 @@
       </c>
       <c r="N63" t="inlineStr"/>
       <c r="O63" t="inlineStr"/>
-      <c r="P63" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q63" s="2" t="n">
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R63" s="2" t="n">
         <v>195</v>
       </c>
     </row>
@@ -4563,10 +4630,11 @@
       </c>
       <c r="N64" t="inlineStr"/>
       <c r="O64" t="inlineStr"/>
-      <c r="P64" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q64" s="2" t="n">
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R64" s="2" t="n">
         <v>585</v>
       </c>
     </row>
@@ -4632,10 +4700,11 @@
       </c>
       <c r="N65" t="inlineStr"/>
       <c r="O65" t="inlineStr"/>
-      <c r="P65" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q65" s="2" t="n">
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R65" s="2" t="n">
         <v>390</v>
       </c>
     </row>
@@ -4689,10 +4758,11 @@
       </c>
       <c r="N66" t="inlineStr"/>
       <c r="O66" t="inlineStr"/>
-      <c r="P66" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q66" s="2" t="n">
+      <c r="P66" t="inlineStr"/>
+      <c r="Q66" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R66" s="2" t="n">
         <v>3315</v>
       </c>
     </row>
@@ -4758,10 +4828,11 @@
       </c>
       <c r="N67" t="inlineStr"/>
       <c r="O67" t="inlineStr"/>
-      <c r="P67" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q67" s="2" t="n">
+      <c r="P67" t="inlineStr"/>
+      <c r="Q67" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R67" s="2" t="n">
         <v>3315</v>
       </c>
     </row>
@@ -4815,10 +4886,11 @@
       </c>
       <c r="N68" t="inlineStr"/>
       <c r="O68" t="inlineStr"/>
-      <c r="P68" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q68" s="2" t="n">
+      <c r="P68" t="inlineStr"/>
+      <c r="Q68" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R68" s="2" t="n">
         <v>2145</v>
       </c>
     </row>
@@ -4884,10 +4956,11 @@
       </c>
       <c r="N69" t="inlineStr"/>
       <c r="O69" t="inlineStr"/>
-      <c r="P69" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q69" s="2" t="n">
+      <c r="P69" t="inlineStr"/>
+      <c r="Q69" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R69" s="2" t="n">
         <v>2145</v>
       </c>
     </row>
@@ -4941,10 +5014,11 @@
       </c>
       <c r="N70" t="inlineStr"/>
       <c r="O70" t="inlineStr"/>
-      <c r="P70" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q70" s="2" t="n">
+      <c r="P70" t="inlineStr"/>
+      <c r="Q70" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R70" s="2" t="n">
         <v>2145</v>
       </c>
     </row>
@@ -5010,10 +5084,11 @@
       </c>
       <c r="N71" t="inlineStr"/>
       <c r="O71" t="inlineStr"/>
-      <c r="P71" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q71" s="2" t="n">
+      <c r="P71" t="inlineStr"/>
+      <c r="Q71" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R71" s="2" t="n">
         <v>2145</v>
       </c>
     </row>
@@ -5067,10 +5142,11 @@
       </c>
       <c r="N72" t="inlineStr"/>
       <c r="O72" t="inlineStr"/>
-      <c r="P72" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q72" s="2" t="n">
+      <c r="P72" t="inlineStr"/>
+      <c r="Q72" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R72" s="2" t="n">
         <v>1950</v>
       </c>
     </row>
@@ -5136,10 +5212,11 @@
       </c>
       <c r="N73" t="inlineStr"/>
       <c r="O73" t="inlineStr"/>
-      <c r="P73" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q73" s="2" t="n">
+      <c r="P73" t="inlineStr"/>
+      <c r="Q73" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R73" s="2" t="n">
         <v>780</v>
       </c>
     </row>
@@ -5205,10 +5282,11 @@
       </c>
       <c r="N74" t="inlineStr"/>
       <c r="O74" t="inlineStr"/>
-      <c r="P74" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q74" s="2" t="n">
+      <c r="P74" t="inlineStr"/>
+      <c r="Q74" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R74" s="2" t="n">
         <v>195</v>
       </c>
     </row>
@@ -5274,10 +5352,11 @@
       </c>
       <c r="N75" t="inlineStr"/>
       <c r="O75" t="inlineStr"/>
-      <c r="P75" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q75" s="2" t="n">
+      <c r="P75" t="inlineStr"/>
+      <c r="Q75" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R75" s="2" t="n">
         <v>585</v>
       </c>
     </row>
@@ -5343,10 +5422,11 @@
       </c>
       <c r="N76" t="inlineStr"/>
       <c r="O76" t="inlineStr"/>
-      <c r="P76" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q76" s="2" t="n">
+      <c r="P76" t="inlineStr"/>
+      <c r="Q76" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R76" s="2" t="n">
         <v>390</v>
       </c>
     </row>
@@ -5400,10 +5480,11 @@
       </c>
       <c r="N77" t="inlineStr"/>
       <c r="O77" t="inlineStr"/>
-      <c r="P77" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q77" s="2" t="n">
+      <c r="P77" t="inlineStr"/>
+      <c r="Q77" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R77" s="2" t="n">
         <v>1950</v>
       </c>
     </row>
@@ -5469,10 +5550,11 @@
       </c>
       <c r="N78" t="inlineStr"/>
       <c r="O78" t="inlineStr"/>
-      <c r="P78" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q78" s="2" t="n">
+      <c r="P78" t="inlineStr"/>
+      <c r="Q78" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R78" s="2" t="n">
         <v>780</v>
       </c>
     </row>
@@ -5538,10 +5620,11 @@
       </c>
       <c r="N79" t="inlineStr"/>
       <c r="O79" t="inlineStr"/>
-      <c r="P79" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q79" s="2" t="n">
+      <c r="P79" t="inlineStr"/>
+      <c r="Q79" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R79" s="2" t="n">
         <v>195</v>
       </c>
     </row>
@@ -5607,10 +5690,11 @@
       </c>
       <c r="N80" t="inlineStr"/>
       <c r="O80" t="inlineStr"/>
-      <c r="P80" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q80" s="2" t="n">
+      <c r="P80" t="inlineStr"/>
+      <c r="Q80" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R80" s="2" t="n">
         <v>585</v>
       </c>
     </row>
@@ -5676,10 +5760,11 @@
       </c>
       <c r="N81" t="inlineStr"/>
       <c r="O81" t="inlineStr"/>
-      <c r="P81" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q81" s="2" t="n">
+      <c r="P81" t="inlineStr"/>
+      <c r="Q81" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R81" s="2" t="n">
         <v>390</v>
       </c>
     </row>
@@ -5733,10 +5818,11 @@
       </c>
       <c r="N82" t="inlineStr"/>
       <c r="O82" t="inlineStr"/>
-      <c r="P82" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q82" s="2" t="n">
+      <c r="P82" t="inlineStr"/>
+      <c r="Q82" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R82" s="2" t="n">
         <v>1755</v>
       </c>
     </row>
@@ -5802,10 +5888,11 @@
       </c>
       <c r="N83" t="inlineStr"/>
       <c r="O83" t="inlineStr"/>
-      <c r="P83" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q83" s="2" t="n">
+      <c r="P83" t="inlineStr"/>
+      <c r="Q83" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R83" s="2" t="n">
         <v>1755</v>
       </c>
     </row>
@@ -5859,10 +5946,11 @@
       </c>
       <c r="N84" t="inlineStr"/>
       <c r="O84" t="inlineStr"/>
-      <c r="P84" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q84" s="2" t="n">
+      <c r="P84" t="inlineStr"/>
+      <c r="Q84" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R84" s="2" t="n">
         <v>585</v>
       </c>
     </row>
@@ -5928,10 +6016,11 @@
       </c>
       <c r="N85" t="inlineStr"/>
       <c r="O85" t="inlineStr"/>
-      <c r="P85" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q85" s="2" t="n">
+      <c r="P85" t="inlineStr"/>
+      <c r="Q85" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R85" s="2" t="n">
         <v>585</v>
       </c>
     </row>
@@ -5985,10 +6074,11 @@
       </c>
       <c r="N86" t="inlineStr"/>
       <c r="O86" t="inlineStr"/>
-      <c r="P86" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q86" s="2" t="n">
+      <c r="P86" t="inlineStr"/>
+      <c r="Q86" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R86" s="2" t="n">
         <v>1365</v>
       </c>
     </row>
@@ -6054,10 +6144,11 @@
       </c>
       <c r="N87" t="inlineStr"/>
       <c r="O87" t="inlineStr"/>
-      <c r="P87" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q87" s="2" t="n">
+      <c r="P87" t="inlineStr"/>
+      <c r="Q87" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R87" s="2" t="n">
         <v>585</v>
       </c>
     </row>
@@ -6123,10 +6214,11 @@
       </c>
       <c r="N88" t="inlineStr"/>
       <c r="O88" t="inlineStr"/>
-      <c r="P88" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q88" s="2" t="n">
+      <c r="P88" t="inlineStr"/>
+      <c r="Q88" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R88" s="2" t="n">
         <v>780</v>
       </c>
     </row>
@@ -6180,10 +6272,11 @@
       </c>
       <c r="N89" t="inlineStr"/>
       <c r="O89" t="inlineStr"/>
-      <c r="P89" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q89" s="2" t="n">
+      <c r="P89" t="inlineStr"/>
+      <c r="Q89" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R89" s="2" t="n">
         <v>1950</v>
       </c>
     </row>
@@ -6249,10 +6342,11 @@
       </c>
       <c r="N90" t="inlineStr"/>
       <c r="O90" t="inlineStr"/>
-      <c r="P90" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q90" s="2" t="n">
+      <c r="P90" t="inlineStr"/>
+      <c r="Q90" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R90" s="2" t="n">
         <v>195</v>
       </c>
     </row>
@@ -6318,10 +6412,11 @@
       </c>
       <c r="N91" t="inlineStr"/>
       <c r="O91" t="inlineStr"/>
-      <c r="P91" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q91" s="2" t="n">
+      <c r="P91" t="inlineStr"/>
+      <c r="Q91" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R91" s="2" t="n">
         <v>195</v>
       </c>
     </row>
@@ -6387,10 +6482,11 @@
       </c>
       <c r="N92" t="inlineStr"/>
       <c r="O92" t="inlineStr"/>
-      <c r="P92" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q92" s="2" t="n">
+      <c r="P92" t="inlineStr"/>
+      <c r="Q92" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R92" s="2" t="n">
         <v>585</v>
       </c>
     </row>
@@ -6456,10 +6552,11 @@
       </c>
       <c r="N93" t="inlineStr"/>
       <c r="O93" t="inlineStr"/>
-      <c r="P93" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q93" s="2" t="n">
+      <c r="P93" t="inlineStr"/>
+      <c r="Q93" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R93" s="2" t="n">
         <v>975</v>
       </c>
     </row>
@@ -6513,10 +6610,11 @@
       </c>
       <c r="N94" t="inlineStr"/>
       <c r="O94" t="inlineStr"/>
-      <c r="P94" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q94" s="2" t="n">
+      <c r="P94" t="inlineStr"/>
+      <c r="Q94" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R94" s="2" t="n">
         <v>2145</v>
       </c>
     </row>
@@ -6582,10 +6680,11 @@
       </c>
       <c r="N95" t="inlineStr"/>
       <c r="O95" t="inlineStr"/>
-      <c r="P95" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q95" s="2" t="n">
+      <c r="P95" t="inlineStr"/>
+      <c r="Q95" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R95" s="2" t="n">
         <v>195</v>
       </c>
     </row>
@@ -6651,10 +6750,11 @@
       </c>
       <c r="N96" t="inlineStr"/>
       <c r="O96" t="inlineStr"/>
-      <c r="P96" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q96" s="2" t="n">
+      <c r="P96" t="inlineStr"/>
+      <c r="Q96" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R96" s="2" t="n">
         <v>585</v>
       </c>
     </row>
@@ -6720,10 +6820,11 @@
       </c>
       <c r="N97" t="inlineStr"/>
       <c r="O97" t="inlineStr"/>
-      <c r="P97" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q97" s="2" t="n">
+      <c r="P97" t="inlineStr"/>
+      <c r="Q97" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R97" s="2" t="n">
         <v>1365</v>
       </c>
     </row>
@@ -6777,10 +6878,11 @@
       </c>
       <c r="N98" t="inlineStr"/>
       <c r="O98" t="inlineStr"/>
-      <c r="P98" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q98" s="2" t="n">
+      <c r="P98" t="inlineStr"/>
+      <c r="Q98" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R98" s="2" t="n">
         <v>780</v>
       </c>
     </row>
@@ -6846,10 +6948,11 @@
       </c>
       <c r="N99" t="inlineStr"/>
       <c r="O99" t="inlineStr"/>
-      <c r="P99" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q99" s="2" t="n">
+      <c r="P99" t="inlineStr"/>
+      <c r="Q99" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R99" s="2" t="n">
         <v>780</v>
       </c>
     </row>
@@ -6903,10 +7006,11 @@
       </c>
       <c r="N100" t="inlineStr"/>
       <c r="O100" t="inlineStr"/>
-      <c r="P100" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q100" s="2" t="n">
+      <c r="P100" t="inlineStr"/>
+      <c r="Q100" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R100" s="2" t="n">
         <v>585</v>
       </c>
     </row>
@@ -6972,10 +7076,11 @@
       </c>
       <c r="N101" t="inlineStr"/>
       <c r="O101" t="inlineStr"/>
-      <c r="P101" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q101" s="2" t="n">
+      <c r="P101" t="inlineStr"/>
+      <c r="Q101" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R101" s="2" t="n">
         <v>390</v>
       </c>
     </row>
@@ -7041,10 +7146,11 @@
       </c>
       <c r="N102" t="inlineStr"/>
       <c r="O102" t="inlineStr"/>
-      <c r="P102" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q102" s="2" t="n">
+      <c r="P102" t="inlineStr"/>
+      <c r="Q102" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R102" s="2" t="n">
         <v>195</v>
       </c>
     </row>
@@ -7098,10 +7204,11 @@
       </c>
       <c r="N103" t="inlineStr"/>
       <c r="O103" t="inlineStr"/>
-      <c r="P103" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q103" s="2" t="n">
+      <c r="P103" t="inlineStr"/>
+      <c r="Q103" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R103" s="2" t="n">
         <v>390</v>
       </c>
     </row>
@@ -7167,10 +7274,11 @@
       </c>
       <c r="N104" t="inlineStr"/>
       <c r="O104" t="inlineStr"/>
-      <c r="P104" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q104" s="2" t="n">
+      <c r="P104" t="inlineStr"/>
+      <c r="Q104" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R104" s="2" t="n">
         <v>390</v>
       </c>
     </row>
@@ -7224,10 +7332,11 @@
       </c>
       <c r="N105" t="inlineStr"/>
       <c r="O105" t="inlineStr"/>
-      <c r="P105" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q105" s="2" t="n">
+      <c r="P105" t="inlineStr"/>
+      <c r="Q105" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R105" s="2" t="n">
         <v>390</v>
       </c>
     </row>
@@ -7293,10 +7402,11 @@
       </c>
       <c r="N106" t="inlineStr"/>
       <c r="O106" t="inlineStr"/>
-      <c r="P106" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q106" s="2" t="n">
+      <c r="P106" t="inlineStr"/>
+      <c r="Q106" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R106" s="2" t="n">
         <v>390</v>
       </c>
     </row>
@@ -7350,10 +7460,11 @@
       </c>
       <c r="N107" t="inlineStr"/>
       <c r="O107" t="inlineStr"/>
-      <c r="P107" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q107" s="2" t="n">
+      <c r="P107" t="inlineStr"/>
+      <c r="Q107" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R107" s="2" t="n">
         <v>390</v>
       </c>
     </row>
@@ -7419,10 +7530,11 @@
       </c>
       <c r="N108" t="inlineStr"/>
       <c r="O108" t="inlineStr"/>
-      <c r="P108" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q108" s="2" t="n">
+      <c r="P108" t="inlineStr"/>
+      <c r="Q108" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R108" s="2" t="n">
         <v>390</v>
       </c>
     </row>
@@ -7476,10 +7588,11 @@
       </c>
       <c r="N109" t="inlineStr"/>
       <c r="O109" t="inlineStr"/>
-      <c r="P109" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q109" s="2" t="n">
+      <c r="P109" t="inlineStr"/>
+      <c r="Q109" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R109" s="2" t="n">
         <v>975</v>
       </c>
     </row>
@@ -7545,10 +7658,11 @@
       </c>
       <c r="N110" t="inlineStr"/>
       <c r="O110" t="inlineStr"/>
-      <c r="P110" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q110" s="2" t="n">
+      <c r="P110" t="inlineStr"/>
+      <c r="Q110" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R110" s="2" t="n">
         <v>975</v>
       </c>
     </row>
@@ -7602,10 +7716,11 @@
       </c>
       <c r="N111" t="inlineStr"/>
       <c r="O111" t="inlineStr"/>
-      <c r="P111" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q111" s="2" t="n">
+      <c r="P111" t="inlineStr"/>
+      <c r="Q111" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R111" s="2" t="n">
         <v>975</v>
       </c>
     </row>
@@ -7671,10 +7786,11 @@
       </c>
       <c r="N112" t="inlineStr"/>
       <c r="O112" t="inlineStr"/>
-      <c r="P112" s="3" t="n">
-        <v>195</v>
-      </c>
-      <c r="Q112" s="2" t="n">
+      <c r="P112" t="inlineStr"/>
+      <c r="Q112" s="3" t="n">
+        <v>195</v>
+      </c>
+      <c r="R112" s="2" t="n">
         <v>975</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update project estimation tool to better handle file exports
Adds an updated export file for project estimations.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 4c2d841a-8e9c-42d2-a44f-f90dc1c78202
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/0e11dc90-618e-44e7-83a8-20eddbc22afb/4c2d841a-8e9c-42d2-a44f-f90dc1c78202/cqhrmiR
</commit_message>
<xml_diff>
--- a/RFP_Brief_ First on SoundCloud 2021 Campaign - Scenario A - Workfront Export.xlsx
+++ b/RFP_Brief_ First on SoundCloud 2021 Campaign - Scenario A - Workfront Export.xlsx
@@ -468,47 +468,47 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Service_Department</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Seniority</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Planned_Hours</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Start_Offset_Days</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Duration_Days</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Dependencies</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Assignee_External_ID</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Service_Department</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
@@ -548,14 +548,16 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+      <c r="L2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
@@ -596,23 +598,23 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" s="2" t="n">
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" s="2" t="n">
         <v>227</v>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="L3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L3" s="2" t="n">
+      <c r="M3" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr">
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
         <is>
           <t>Core/T2_MediumVolume</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
       <c r="Q3" s="3" t="n">
         <v>195</v>
       </c>
@@ -654,21 +656,21 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" s="2" t="n">
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="L4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L4" s="2" t="n">
+      <c r="M4" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>1.1</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" s="3" t="n">
@@ -714,31 +716,31 @@
           <t>Accessibility Audit</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
         <is>
           <t>Accessibility Specialist</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J5" s="2" t="n">
+      <c r="K5" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="L5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L5" s="2" t="n">
+      <c r="M5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>1.1.1</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" s="3" t="n">
@@ -784,31 +786,31 @@
           <t>Accessibility QA</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
         <is>
           <t>QA Engineer</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="K6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="L6" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L6" s="2" t="n">
+      <c r="M6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>1.1.1.1</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" s="3" t="n">
@@ -854,31 +856,31 @@
           <t>Code Review</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
         <is>
           <t>Frontend Engineer</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="K7" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="L7" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="L7" s="2" t="n">
+      <c r="M7" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>1.1.1.2</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" s="3" t="n">
@@ -922,21 +924,21 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" s="2" t="n">
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="L8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L8" s="2" t="n">
+      <c r="M8" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>1.1.1</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" s="3" t="n">
@@ -982,31 +984,31 @@
           <t>Analytics Audit</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
         <is>
           <t>Business Analyst</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="K9" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="L9" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L9" s="2" t="n">
+      <c r="M9" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>1.1.2</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" s="3" t="n">
@@ -1050,21 +1052,21 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" s="2" t="n">
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="L10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L10" s="2" t="n">
+      <c r="M10" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>1.1.2</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" s="3" t="n">
@@ -1110,31 +1112,31 @@
           <t>Documentation</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
         <is>
           <t>Business Analyst</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J11" s="2" t="n">
+      <c r="K11" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="L11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L11" s="2" t="n">
+      <c r="M11" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>1.1.3</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" s="3" t="n">
@@ -1178,21 +1180,21 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" s="2" t="n">
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="L12" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="L12" s="2" t="n">
+      <c r="M12" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>1.1.3</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" s="3" t="n">
@@ -1238,31 +1240,31 @@
           <t>Design Consult</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
         <is>
           <t>UI Designer</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
-      </c>
-      <c r="J13" s="2" t="n">
-        <v>3</v>
       </c>
       <c r="K13" s="2" t="n">
         <v>3</v>
       </c>
       <c r="L13" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M13" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>1.1.4</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" s="3" t="n">
@@ -1308,31 +1310,31 @@
           <t>Accessibility QA</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
         <is>
           <t>QA Engineer</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J14" s="2" t="n">
+      <c r="K14" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="K14" s="2" t="n">
+      <c r="L14" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L14" s="2" t="n">
+      <c r="M14" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>1.1.4.1</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" s="3" t="n">
@@ -1378,31 +1380,31 @@
           <t>Code Review</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
         <is>
           <t>Backend Engineer</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="K15" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="K15" s="2" t="n">
+      <c r="L15" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="L15" s="2" t="n">
+      <c r="M15" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>1.1.4.2</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" s="3" t="n">
@@ -1446,21 +1448,21 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" s="2" t="n">
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="K16" s="2" t="n">
+      <c r="L16" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="L16" s="2" t="n">
+      <c r="M16" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>1.1.4</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" s="3" t="n">
@@ -1506,31 +1508,31 @@
           <t>Design Consult</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
         <is>
           <t>UI Designer</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
-      </c>
-      <c r="J17" s="2" t="n">
-        <v>3</v>
       </c>
       <c r="K17" s="2" t="n">
         <v>3</v>
       </c>
       <c r="L17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M17" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>1.1.5</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" s="3" t="n">
@@ -1576,31 +1578,31 @@
           <t>Accessibility QA</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
         <is>
           <t>QA Engineer</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J18" s="2" t="n">
+      <c r="K18" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="K18" s="2" t="n">
+      <c r="L18" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L18" s="2" t="n">
+      <c r="M18" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>1.1.5.1</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" s="3" t="n">
@@ -1646,31 +1648,31 @@
           <t>Code Review</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
         <is>
           <t>Backend Engineer</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J19" s="2" t="n">
+      <c r="K19" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="K19" s="2" t="n">
+      <c r="L19" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="L19" s="2" t="n">
+      <c r="M19" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>1.1.5.2</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" s="3" t="n">
@@ -1714,21 +1716,21 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" s="2" t="n">
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="K20" s="2" t="n">
+      <c r="L20" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L20" s="2" t="n">
+      <c r="M20" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>1.1.5</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" s="3" t="n">
@@ -1774,31 +1776,31 @@
           <t>QA Cycle</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
         <is>
           <t>QA Engineer</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J21" s="2" t="n">
+      <c r="K21" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K21" s="2" t="n">
+      <c r="L21" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L21" s="2" t="n">
+      <c r="M21" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>1.1.6</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" s="3" t="n">
@@ -1844,31 +1846,31 @@
           <t>Define &amp; Configure Goals</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
         <is>
           <t>Data/Analytics Engineer</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J22" s="2" t="n">
+      <c r="K22" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K22" s="2" t="n">
+      <c r="L22" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="L22" s="2" t="n">
+      <c r="M22" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>1.1.6.1</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" s="3" t="n">
@@ -1912,21 +1914,21 @@
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" s="2" t="n">
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="K23" s="2" t="n">
+      <c r="L23" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L23" s="2" t="n">
+      <c r="M23" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>1.1.6</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" s="3" t="n">
@@ -1972,31 +1974,31 @@
           <t>QA Cycle</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
         <is>
           <t>QA Engineer</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J24" s="2" t="n">
+      <c r="K24" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K24" s="2" t="n">
+      <c r="L24" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L24" s="2" t="n">
+      <c r="M24" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>1.1.7</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" s="3" t="n">
@@ -2042,31 +2044,31 @@
           <t>Event Schema &amp; Tagging</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
         <is>
           <t>Data/Analytics Engineer</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J25" s="2" t="n">
+      <c r="K25" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K25" s="2" t="n">
+      <c r="L25" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="L25" s="2" t="n">
+      <c r="M25" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>1.1.7.1</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" s="3" t="n">
@@ -2110,21 +2112,21 @@
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" s="2" t="n">
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="K26" s="2" t="n">
+      <c r="L26" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L26" s="2" t="n">
+      <c r="M26" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>1.1.7</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" s="3" t="n">
@@ -2170,31 +2172,31 @@
           <t>Spec QA</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
         <is>
           <t>QA Engineer</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J27" s="2" t="n">
+      <c r="K27" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K27" s="2" t="n">
+      <c r="L27" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L27" s="2" t="n">
+      <c r="M27" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>1.1.8</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" s="3" t="n">
@@ -2240,31 +2242,31 @@
           <t>Pixel Setup (GTM)</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
         <is>
           <t>Data/Analytics Engineer</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J28" s="2" t="n">
+      <c r="K28" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K28" s="2" t="n">
+      <c r="L28" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="L28" s="2" t="n">
+      <c r="M28" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="N28" t="inlineStr">
         <is>
           <t>1.1.8.1</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" s="3" t="n">
@@ -2308,21 +2310,21 @@
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" s="2" t="n">
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="K29" s="2" t="n">
+      <c r="L29" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L29" s="2" t="n">
+      <c r="M29" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="N29" t="inlineStr">
         <is>
           <t>1.1.8</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" s="3" t="n">
@@ -2368,31 +2370,31 @@
           <t>QA Cycle</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
         <is>
           <t>QA Engineer</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J30" s="2" t="n">
+      <c r="K30" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K30" s="2" t="n">
+      <c r="L30" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L30" s="2" t="n">
+      <c r="M30" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>1.1.9</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" s="3" t="n">
@@ -2438,31 +2440,31 @@
           <t>Migrate UA Goals → GA4 Conversions</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
         <is>
           <t>Data/Analytics Engineer</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J31" s="2" t="n">
+      <c r="K31" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K31" s="2" t="n">
+      <c r="L31" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="L31" s="2" t="n">
+      <c r="M31" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>1.1.9.1</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" s="3" t="n">
@@ -2506,21 +2508,21 @@
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" s="2" t="n">
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="K32" s="2" t="n">
+      <c r="L32" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L32" s="2" t="n">
+      <c r="M32" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="N32" t="inlineStr">
         <is>
           <t>1.1.9</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" s="3" t="n">
@@ -2566,31 +2568,31 @@
           <t>QA Cycle</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
         <is>
           <t>QA Engineer</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="J33" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J33" s="2" t="n">
+      <c r="K33" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K33" s="2" t="n">
+      <c r="L33" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L33" s="2" t="n">
+      <c r="M33" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="N33" t="inlineStr">
         <is>
           <t>1.1.10</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" s="3" t="n">
@@ -2636,31 +2638,31 @@
           <t>Implement Tags/Events</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
         <is>
           <t>Data/Analytics Engineer</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J34" s="2" t="n">
+      <c r="K34" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K34" s="2" t="n">
+      <c r="L34" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="L34" s="2" t="n">
+      <c r="M34" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="N34" t="inlineStr">
         <is>
           <t>1.1.10.1</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" s="3" t="n">
@@ -2704,21 +2706,21 @@
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" s="2" t="n">
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="K35" s="2" t="n">
+      <c r="L35" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L35" s="2" t="n">
+      <c r="M35" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="N35" t="inlineStr">
         <is>
           <t>1.1.10</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" s="3" t="n">
@@ -2764,31 +2766,31 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
         <is>
           <t>QA Engineer</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="J36" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J36" s="2" t="n">
+      <c r="K36" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K36" s="2" t="n">
+      <c r="L36" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L36" s="2" t="n">
+      <c r="M36" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="N36" t="inlineStr">
         <is>
           <t>1.1.11</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" s="3" t="n">
@@ -2834,31 +2836,31 @@
           <t>Event Config</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
         <is>
           <t>Data/Analytics Engineer</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J37" s="2" t="n">
+      <c r="K37" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K37" s="2" t="n">
+      <c r="L37" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="L37" s="2" t="n">
+      <c r="M37" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M37" t="inlineStr">
+      <c r="N37" t="inlineStr">
         <is>
           <t>1.1.11.1</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" s="3" t="n">
@@ -2902,21 +2904,21 @@
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" s="2" t="n">
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K38" s="2" t="n">
+      <c r="L38" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L38" s="2" t="n">
+      <c r="M38" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M38" t="inlineStr">
+      <c r="N38" t="inlineStr">
         <is>
           <t>1.1.11</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" s="3" t="n">
@@ -2962,31 +2964,31 @@
           <t>Publish &amp; Smoke Test</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
         <is>
           <t>QA Engineer</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J39" s="2" t="n">
+      <c r="K39" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K39" s="2" t="n">
+      <c r="L39" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L39" s="2" t="n">
+      <c r="M39" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M39" t="inlineStr">
+      <c r="N39" t="inlineStr">
         <is>
           <t>1.1.12</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" s="3" t="n">
@@ -3030,21 +3032,21 @@
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr"/>
-      <c r="J40" s="2" t="n">
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K40" s="2" t="n">
+      <c r="L40" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L40" s="2" t="n">
+      <c r="M40" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="M40" t="inlineStr">
+      <c r="N40" t="inlineStr">
         <is>
           <t>1.1.12</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" s="3" t="n">
@@ -3090,31 +3092,31 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
         <is>
           <t>QA Engineer</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="J41" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J41" s="2" t="n">
+      <c r="K41" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K41" s="2" t="n">
+      <c r="L41" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L41" s="2" t="n">
+      <c r="M41" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="N41" t="inlineStr">
         <is>
           <t>1.1.13</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" s="3" t="n">
@@ -3160,31 +3162,31 @@
           <t>Cross-domain Config</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
         <is>
           <t>Data/Analytics Engineer</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="J42" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J42" s="2" t="n">
+      <c r="K42" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K42" s="2" t="n">
+      <c r="L42" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="L42" s="2" t="n">
+      <c r="M42" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="N42" t="inlineStr">
         <is>
           <t>1.1.13.1</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" s="3" t="n">
@@ -3228,21 +3230,21 @@
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr"/>
-      <c r="J43" s="2" t="n">
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K43" s="2" t="n">
+      <c r="L43" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L43" s="2" t="n">
+      <c r="M43" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="N43" t="inlineStr">
         <is>
           <t>1.1.13</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr"/>
       <c r="Q43" s="3" t="n">
@@ -3288,31 +3290,31 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
         <is>
           <t>QA Engineer</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="J44" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J44" s="2" t="n">
+      <c r="K44" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K44" s="2" t="n">
+      <c r="L44" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L44" s="2" t="n">
+      <c r="M44" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M44" t="inlineStr">
+      <c r="N44" t="inlineStr">
         <is>
           <t>1.1.14</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" s="3" t="n">
@@ -3358,31 +3360,31 @@
           <t>Ecommerce Data Layer</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
         <is>
           <t>Data/Analytics Engineer</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="J45" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J45" s="2" t="n">
+      <c r="K45" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K45" s="2" t="n">
+      <c r="L45" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="L45" s="2" t="n">
+      <c r="M45" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M45" t="inlineStr">
+      <c r="N45" t="inlineStr">
         <is>
           <t>1.1.14.1</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr"/>
       <c r="Q45" s="3" t="n">
@@ -3426,21 +3428,21 @@
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr"/>
-      <c r="J46" s="2" t="n">
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="K46" s="2" t="n">
+      <c r="L46" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L46" s="2" t="n">
+      <c r="M46" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="M46" t="inlineStr">
+      <c r="N46" t="inlineStr">
         <is>
           <t>1.1.14</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr"/>
       <c r="Q46" s="3" t="n">
@@ -3486,31 +3488,31 @@
           <t>QA Cycle</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
         <is>
           <t>QA Engineer</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="J47" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J47" s="2" t="n">
+      <c r="K47" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K47" s="2" t="n">
+      <c r="L47" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L47" s="2" t="n">
+      <c r="M47" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M47" t="inlineStr">
+      <c r="N47" t="inlineStr">
         <is>
           <t>1.1.15</t>
         </is>
       </c>
-      <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr"/>
       <c r="Q47" s="3" t="n">
@@ -3556,31 +3558,31 @@
           <t>GA4 Property Setup</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
         <is>
           <t>Data/Analytics Engineer</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
+      <c r="J48" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J48" s="2" t="n">
+      <c r="K48" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K48" s="2" t="n">
+      <c r="L48" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="L48" s="2" t="n">
+      <c r="M48" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M48" t="inlineStr">
+      <c r="N48" t="inlineStr">
         <is>
           <t>1.1.15.1</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr"/>
       <c r="Q48" s="3" t="n">
@@ -3620,27 +3622,27 @@
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr"/>
-      <c r="J49" s="2" t="n">
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" s="2" t="n">
         <v>188</v>
       </c>
-      <c r="K49" s="2" t="n">
+      <c r="L49" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="L49" s="2" t="n">
+      <c r="M49" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="M49" t="inlineStr">
+      <c r="N49" t="inlineStr">
         <is>
           <t>1.1</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr">
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr">
         <is>
           <t>Core/T2_MediumVolume</t>
         </is>
       </c>
-      <c r="P49" t="inlineStr"/>
       <c r="Q49" s="3" t="n">
         <v>195</v>
       </c>
@@ -3682,21 +3684,21 @@
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr"/>
-      <c r="J50" s="2" t="n">
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K50" s="2" t="n">
+      <c r="L50" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="L50" s="2" t="n">
+      <c r="M50" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M50" t="inlineStr">
+      <c r="N50" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr"/>
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr"/>
       <c r="Q50" s="3" t="n">
@@ -3742,31 +3744,31 @@
           <t>Rights/License Research</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
         <is>
           <t>Producer</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
+      <c r="J51" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J51" s="2" t="n">
+      <c r="K51" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K51" s="2" t="n">
+      <c r="L51" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="L51" s="2" t="n">
+      <c r="M51" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M51" t="inlineStr">
+      <c r="N51" t="inlineStr">
         <is>
           <t>1.2.1</t>
         </is>
       </c>
-      <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr"/>
       <c r="Q51" s="3" t="n">
@@ -3812,31 +3814,31 @@
           <t>Usage Notes</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
         <is>
           <t>Account Manager</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
+      <c r="J52" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J52" s="2" t="n">
+      <c r="K52" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K52" s="2" t="n">
+      <c r="L52" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="L52" s="2" t="n">
+      <c r="M52" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M52" t="inlineStr">
+      <c r="N52" t="inlineStr">
         <is>
           <t>1.2.1.1</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr"/>
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr"/>
       <c r="Q52" s="3" t="n">
@@ -3880,21 +3882,21 @@
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr"/>
-      <c r="J53" s="2" t="n">
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="K53" s="2" t="n">
+      <c r="L53" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="L53" s="2" t="n">
+      <c r="M53" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="M53" t="inlineStr">
+      <c r="N53" t="inlineStr">
         <is>
           <t>1.2.1</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr"/>
       <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr"/>
       <c r="Q53" s="3" t="n">
@@ -3940,31 +3942,31 @@
           <t>Script Polish</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
         <is>
           <t>Copywriter</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
+      <c r="J54" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J54" s="2" t="n">
+      <c r="K54" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K54" s="2" t="n">
+      <c r="L54" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="L54" s="2" t="n">
+      <c r="M54" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="M54" t="inlineStr">
+      <c r="N54" t="inlineStr">
         <is>
           <t>1.2.2</t>
         </is>
       </c>
-      <c r="N54" t="inlineStr"/>
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr"/>
       <c r="Q54" s="3" t="n">
@@ -4010,31 +4012,31 @@
           <t>VO Session</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr">
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
         <is>
           <t>Sound Designer</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr">
+      <c r="J55" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J55" s="2" t="n">
+      <c r="K55" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K55" s="2" t="n">
+      <c r="L55" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="L55" s="2" t="n">
+      <c r="M55" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M55" t="inlineStr">
+      <c r="N55" t="inlineStr">
         <is>
           <t>1.2.2.1</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr"/>
       <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr"/>
       <c r="Q55" s="3" t="n">
@@ -4078,21 +4080,21 @@
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr"/>
-      <c r="J56" s="2" t="n">
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="K56" s="2" t="n">
+      <c r="L56" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="L56" s="2" t="n">
+      <c r="M56" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="M56" t="inlineStr">
+      <c r="N56" t="inlineStr">
         <is>
           <t>1.2.2</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr"/>
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr"/>
       <c r="Q56" s="3" t="n">
@@ -4138,31 +4140,31 @@
           <t>Client Review &amp; Revisions</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
         <is>
           <t>Editor</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr">
+      <c r="J57" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J57" s="2" t="n">
+      <c r="K57" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="K57" s="2" t="n">
+      <c r="L57" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="L57" s="2" t="n">
+      <c r="M57" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="M57" t="inlineStr">
+      <c r="N57" t="inlineStr">
         <is>
           <t>1.2.3</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr"/>
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr"/>
       <c r="Q57" s="3" t="n">
@@ -4206,21 +4208,21 @@
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr"/>
-      <c r="J58" s="2" t="n">
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="K58" s="2" t="n">
+      <c r="L58" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="L58" s="2" t="n">
+      <c r="M58" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="M58" t="inlineStr">
+      <c r="N58" t="inlineStr">
         <is>
           <t>1.2.3</t>
         </is>
       </c>
-      <c r="N58" t="inlineStr"/>
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr"/>
       <c r="Q58" s="3" t="n">
@@ -4266,31 +4268,31 @@
           <t>Client Review &amp; Revisions</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr">
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
         <is>
           <t>Editor</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr">
+      <c r="J59" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J59" s="2" t="n">
+      <c r="K59" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="K59" s="2" t="n">
+      <c r="L59" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="L59" s="2" t="n">
+      <c r="M59" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="M59" t="inlineStr">
+      <c r="N59" t="inlineStr">
         <is>
           <t>1.2.4</t>
         </is>
       </c>
-      <c r="N59" t="inlineStr"/>
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr"/>
       <c r="Q59" s="3" t="n">
@@ -4334,21 +4336,21 @@
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr"/>
-      <c r="J60" s="2" t="n">
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="K60" s="2" t="n">
+      <c r="L60" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="L60" s="2" t="n">
+      <c r="M60" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="M60" t="inlineStr">
+      <c r="N60" t="inlineStr">
         <is>
           <t>1.2.4</t>
         </is>
       </c>
-      <c r="N60" t="inlineStr"/>
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr"/>
       <c r="Q60" s="3" t="n">
@@ -4394,31 +4396,31 @@
           <t>VO Edit</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr">
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
         <is>
           <t>Editor</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr">
+      <c r="J61" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J61" s="2" t="n">
+      <c r="K61" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="K61" s="2" t="n">
+      <c r="L61" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="L61" s="2" t="n">
+      <c r="M61" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="M61" t="inlineStr">
+      <c r="N61" t="inlineStr">
         <is>
           <t>1.2.5</t>
         </is>
       </c>
-      <c r="N61" t="inlineStr"/>
       <c r="O61" t="inlineStr"/>
       <c r="P61" t="inlineStr"/>
       <c r="Q61" s="3" t="n">
@@ -4464,31 +4466,31 @@
           <t>Mix</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr">
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
         <is>
           <t>Sound Designer</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr">
+      <c r="J62" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J62" s="2" t="n">
+      <c r="K62" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K62" s="2" t="n">
+      <c r="L62" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="L62" s="2" t="n">
+      <c r="M62" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M62" t="inlineStr">
+      <c r="N62" t="inlineStr">
         <is>
           <t>1.2.5.1</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr"/>
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr"/>
       <c r="Q62" s="3" t="n">
@@ -4534,31 +4536,31 @@
           <t>Internal Review &amp; Critique</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr">
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
         <is>
           <t>Producer</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr">
+      <c r="J63" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J63" s="2" t="n">
+      <c r="K63" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K63" s="2" t="n">
+      <c r="L63" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="L63" s="2" t="n">
+      <c r="M63" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M63" t="inlineStr">
+      <c r="N63" t="inlineStr">
         <is>
           <t>1.2.5.2</t>
         </is>
       </c>
-      <c r="N63" t="inlineStr"/>
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr"/>
       <c r="Q63" s="3" t="n">
@@ -4604,31 +4606,31 @@
           <t>Client Review &amp; Revisions</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr">
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
         <is>
           <t>Account Manager</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr">
+      <c r="J64" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J64" s="2" t="n">
+      <c r="K64" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K64" s="2" t="n">
+      <c r="L64" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="L64" s="2" t="n">
+      <c r="M64" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M64" t="inlineStr">
+      <c r="N64" t="inlineStr">
         <is>
           <t>1.2.5.3</t>
         </is>
       </c>
-      <c r="N64" t="inlineStr"/>
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr"/>
       <c r="Q64" s="3" t="n">
@@ -4674,31 +4676,31 @@
           <t>Final Packaging</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr">
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
         <is>
           <t>Designer</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr">
+      <c r="J65" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J65" s="2" t="n">
+      <c r="K65" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K65" s="2" t="n">
+      <c r="L65" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="L65" s="2" t="n">
+      <c r="M65" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M65" t="inlineStr">
+      <c r="N65" t="inlineStr">
         <is>
           <t>1.2.5.4</t>
         </is>
       </c>
-      <c r="N65" t="inlineStr"/>
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr"/>
       <c r="Q65" s="3" t="n">
@@ -4742,21 +4744,21 @@
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr"/>
-      <c r="J66" s="2" t="n">
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="K66" s="2" t="n">
+      <c r="L66" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="L66" s="2" t="n">
+      <c r="M66" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="M66" t="inlineStr">
+      <c r="N66" t="inlineStr">
         <is>
           <t>1.2.5</t>
         </is>
       </c>
-      <c r="N66" t="inlineStr"/>
       <c r="O66" t="inlineStr"/>
       <c r="P66" t="inlineStr"/>
       <c r="Q66" s="3" t="n">
@@ -4802,31 +4804,31 @@
           <t>Client Review &amp; Revisions</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr">
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
         <is>
           <t>Editor</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr">
+      <c r="J67" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J67" s="2" t="n">
+      <c r="K67" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="K67" s="2" t="n">
+      <c r="L67" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="L67" s="2" t="n">
+      <c r="M67" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="M67" t="inlineStr">
+      <c r="N67" t="inlineStr">
         <is>
           <t>1.2.6</t>
         </is>
       </c>
-      <c r="N67" t="inlineStr"/>
       <c r="O67" t="inlineStr"/>
       <c r="P67" t="inlineStr"/>
       <c r="Q67" s="3" t="n">
@@ -4870,21 +4872,21 @@
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr"/>
-      <c r="J68" s="2" t="n">
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="K68" s="2" t="n">
+      <c r="L68" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="L68" s="2" t="n">
+      <c r="M68" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M68" t="inlineStr">
+      <c r="N68" t="inlineStr">
         <is>
           <t>1.2.6</t>
         </is>
       </c>
-      <c r="N68" t="inlineStr"/>
       <c r="O68" t="inlineStr"/>
       <c r="P68" t="inlineStr"/>
       <c r="Q68" s="3" t="n">
@@ -4930,31 +4932,31 @@
           <t>Client Review &amp; Revisions</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr">
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
         <is>
           <t>Colorist</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr">
+      <c r="J69" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J69" s="2" t="n">
+      <c r="K69" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="K69" s="2" t="n">
+      <c r="L69" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="L69" s="2" t="n">
+      <c r="M69" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M69" t="inlineStr">
+      <c r="N69" t="inlineStr">
         <is>
           <t>1.2.7</t>
         </is>
       </c>
-      <c r="N69" t="inlineStr"/>
       <c r="O69" t="inlineStr"/>
       <c r="P69" t="inlineStr"/>
       <c r="Q69" s="3" t="n">
@@ -4998,21 +5000,21 @@
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr"/>
-      <c r="J70" s="2" t="n">
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="K70" s="2" t="n">
+      <c r="L70" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="L70" s="2" t="n">
+      <c r="M70" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M70" t="inlineStr">
+      <c r="N70" t="inlineStr">
         <is>
           <t>1.2.7</t>
         </is>
       </c>
-      <c r="N70" t="inlineStr"/>
       <c r="O70" t="inlineStr"/>
       <c r="P70" t="inlineStr"/>
       <c r="Q70" s="3" t="n">
@@ -5058,31 +5060,31 @@
           <t>Client Review &amp; Revisions</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr">
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
         <is>
           <t>Colorist</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr">
+      <c r="J71" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J71" s="2" t="n">
+      <c r="K71" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="K71" s="2" t="n">
+      <c r="L71" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="L71" s="2" t="n">
+      <c r="M71" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M71" t="inlineStr">
+      <c r="N71" t="inlineStr">
         <is>
           <t>1.2.8</t>
         </is>
       </c>
-      <c r="N71" t="inlineStr"/>
       <c r="O71" t="inlineStr"/>
       <c r="P71" t="inlineStr"/>
       <c r="Q71" s="3" t="n">
@@ -5126,21 +5128,21 @@
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr"/>
-      <c r="J72" s="2" t="n">
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="K72" s="2" t="n">
+      <c r="L72" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="L72" s="2" t="n">
+      <c r="M72" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="M72" t="inlineStr">
+      <c r="N72" t="inlineStr">
         <is>
           <t>1.2.8</t>
         </is>
       </c>
-      <c r="N72" t="inlineStr"/>
       <c r="O72" t="inlineStr"/>
       <c r="P72" t="inlineStr"/>
       <c r="Q72" s="3" t="n">
@@ -5186,31 +5188,31 @@
           <t>Retouch</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr">
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
         <is>
           <t>Retoucher</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr">
+      <c r="J73" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J73" s="2" t="n">
+      <c r="K73" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K73" s="2" t="n">
+      <c r="L73" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="L73" s="2" t="n">
+      <c r="M73" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M73" t="inlineStr">
+      <c r="N73" t="inlineStr">
         <is>
           <t>1.2.9</t>
         </is>
       </c>
-      <c r="N73" t="inlineStr"/>
       <c r="O73" t="inlineStr"/>
       <c r="P73" t="inlineStr"/>
       <c r="Q73" s="3" t="n">
@@ -5256,31 +5258,31 @@
           <t>Internal Review &amp; Critique</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr">
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
         <is>
           <t>Producer</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr">
+      <c r="J74" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J74" s="2" t="n">
+      <c r="K74" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K74" s="2" t="n">
+      <c r="L74" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="L74" s="2" t="n">
+      <c r="M74" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M74" t="inlineStr">
+      <c r="N74" t="inlineStr">
         <is>
           <t>1.2.9.1</t>
         </is>
       </c>
-      <c r="N74" t="inlineStr"/>
       <c r="O74" t="inlineStr"/>
       <c r="P74" t="inlineStr"/>
       <c r="Q74" s="3" t="n">
@@ -5326,31 +5328,31 @@
           <t>Client Review &amp; Revisions</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr">
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
         <is>
           <t>Account Manager</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr">
+      <c r="J75" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J75" s="2" t="n">
+      <c r="K75" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K75" s="2" t="n">
+      <c r="L75" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="L75" s="2" t="n">
+      <c r="M75" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M75" t="inlineStr">
+      <c r="N75" t="inlineStr">
         <is>
           <t>1.2.9.2</t>
         </is>
       </c>
-      <c r="N75" t="inlineStr"/>
       <c r="O75" t="inlineStr"/>
       <c r="P75" t="inlineStr"/>
       <c r="Q75" s="3" t="n">
@@ -5396,31 +5398,31 @@
           <t>Final Packaging</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr">
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
         <is>
           <t>Designer</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr">
+      <c r="J76" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J76" s="2" t="n">
+      <c r="K76" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K76" s="2" t="n">
+      <c r="L76" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="L76" s="2" t="n">
+      <c r="M76" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M76" t="inlineStr">
+      <c r="N76" t="inlineStr">
         <is>
           <t>1.2.9.3</t>
         </is>
       </c>
-      <c r="N76" t="inlineStr"/>
       <c r="O76" t="inlineStr"/>
       <c r="P76" t="inlineStr"/>
       <c r="Q76" s="3" t="n">
@@ -5464,21 +5466,21 @@
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr"/>
-      <c r="J77" s="2" t="n">
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="K77" s="2" t="n">
+      <c r="L77" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="L77" s="2" t="n">
+      <c r="M77" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="M77" t="inlineStr">
+      <c r="N77" t="inlineStr">
         <is>
           <t>1.2.9</t>
         </is>
       </c>
-      <c r="N77" t="inlineStr"/>
       <c r="O77" t="inlineStr"/>
       <c r="P77" t="inlineStr"/>
       <c r="Q77" s="3" t="n">
@@ -5524,31 +5526,31 @@
           <t>Retouch</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr">
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
         <is>
           <t>Retoucher</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr">
+      <c r="J78" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J78" s="2" t="n">
+      <c r="K78" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K78" s="2" t="n">
+      <c r="L78" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="L78" s="2" t="n">
+      <c r="M78" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M78" t="inlineStr">
+      <c r="N78" t="inlineStr">
         <is>
           <t>1.2.10</t>
         </is>
       </c>
-      <c r="N78" t="inlineStr"/>
       <c r="O78" t="inlineStr"/>
       <c r="P78" t="inlineStr"/>
       <c r="Q78" s="3" t="n">
@@ -5594,31 +5596,31 @@
           <t>Internal Review &amp; Critique</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr">
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
         <is>
           <t>Producer</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr">
+      <c r="J79" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J79" s="2" t="n">
+      <c r="K79" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K79" s="2" t="n">
+      <c r="L79" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="L79" s="2" t="n">
+      <c r="M79" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M79" t="inlineStr">
+      <c r="N79" t="inlineStr">
         <is>
           <t>1.2.10.1</t>
         </is>
       </c>
-      <c r="N79" t="inlineStr"/>
       <c r="O79" t="inlineStr"/>
       <c r="P79" t="inlineStr"/>
       <c r="Q79" s="3" t="n">
@@ -5664,31 +5666,31 @@
           <t>Client Review &amp; Revisions</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr">
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr">
         <is>
           <t>Account Manager</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr">
+      <c r="J80" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J80" s="2" t="n">
+      <c r="K80" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K80" s="2" t="n">
+      <c r="L80" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="L80" s="2" t="n">
+      <c r="M80" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M80" t="inlineStr">
+      <c r="N80" t="inlineStr">
         <is>
           <t>1.2.10.2</t>
         </is>
       </c>
-      <c r="N80" t="inlineStr"/>
       <c r="O80" t="inlineStr"/>
       <c r="P80" t="inlineStr"/>
       <c r="Q80" s="3" t="n">
@@ -5734,31 +5736,31 @@
           <t>Final Packaging</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr">
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr">
         <is>
           <t>Designer</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr">
+      <c r="J81" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J81" s="2" t="n">
+      <c r="K81" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K81" s="2" t="n">
+      <c r="L81" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="L81" s="2" t="n">
+      <c r="M81" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M81" t="inlineStr">
+      <c r="N81" t="inlineStr">
         <is>
           <t>1.2.10.3</t>
         </is>
       </c>
-      <c r="N81" t="inlineStr"/>
       <c r="O81" t="inlineStr"/>
       <c r="P81" t="inlineStr"/>
       <c r="Q81" s="3" t="n">
@@ -5802,21 +5804,21 @@
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr"/>
       <c r="I82" t="inlineStr"/>
-      <c r="J82" s="2" t="n">
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="K82" s="2" t="n">
+      <c r="L82" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="L82" s="2" t="n">
+      <c r="M82" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M82" t="inlineStr">
+      <c r="N82" t="inlineStr">
         <is>
           <t>1.2.10</t>
         </is>
       </c>
-      <c r="N82" t="inlineStr"/>
       <c r="O82" t="inlineStr"/>
       <c r="P82" t="inlineStr"/>
       <c r="Q82" s="3" t="n">
@@ -5862,31 +5864,31 @@
           <t>Client Review &amp; Revisions</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr">
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr">
         <is>
           <t>Designer</t>
         </is>
       </c>
-      <c r="I83" t="inlineStr">
+      <c r="J83" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J83" s="2" t="n">
+      <c r="K83" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="K83" s="2" t="n">
+      <c r="L83" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="L83" s="2" t="n">
+      <c r="M83" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M83" t="inlineStr">
+      <c r="N83" t="inlineStr">
         <is>
           <t>1.2.11</t>
         </is>
       </c>
-      <c r="N83" t="inlineStr"/>
       <c r="O83" t="inlineStr"/>
       <c r="P83" t="inlineStr"/>
       <c r="Q83" s="3" t="n">
@@ -5930,21 +5932,21 @@
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr"/>
       <c r="I84" t="inlineStr"/>
-      <c r="J84" s="2" t="n">
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K84" s="2" t="n">
+      <c r="L84" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="L84" s="2" t="n">
+      <c r="M84" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M84" t="inlineStr">
+      <c r="N84" t="inlineStr">
         <is>
           <t>1.2.11</t>
         </is>
       </c>
-      <c r="N84" t="inlineStr"/>
       <c r="O84" t="inlineStr"/>
       <c r="P84" t="inlineStr"/>
       <c r="Q84" s="3" t="n">
@@ -5990,31 +5992,31 @@
           <t>Music Search &amp; License</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr">
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr">
         <is>
           <t>Sound Designer</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr">
+      <c r="J85" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J85" s="2" t="n">
+      <c r="K85" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K85" s="2" t="n">
+      <c r="L85" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="L85" s="2" t="n">
+      <c r="M85" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M85" t="inlineStr">
+      <c r="N85" t="inlineStr">
         <is>
           <t>1.2.12</t>
         </is>
       </c>
-      <c r="N85" t="inlineStr"/>
       <c r="O85" t="inlineStr"/>
       <c r="P85" t="inlineStr"/>
       <c r="Q85" s="3" t="n">
@@ -6058,21 +6060,21 @@
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr"/>
-      <c r="J86" s="2" t="n">
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="K86" s="2" t="n">
+      <c r="L86" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="L86" s="2" t="n">
+      <c r="M86" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M86" t="inlineStr">
+      <c r="N86" t="inlineStr">
         <is>
           <t>1.2.12</t>
         </is>
       </c>
-      <c r="N86" t="inlineStr"/>
       <c r="O86" t="inlineStr"/>
       <c r="P86" t="inlineStr"/>
       <c r="Q86" s="3" t="n">
@@ -6118,31 +6120,31 @@
           <t>QA (Tech &amp; Content)</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr">
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr">
         <is>
           <t>QA Specialist</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr">
+      <c r="J87" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J87" s="2" t="n">
+      <c r="K87" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K87" s="2" t="n">
+      <c r="L87" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="L87" s="2" t="n">
+      <c r="M87" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M87" t="inlineStr">
+      <c r="N87" t="inlineStr">
         <is>
           <t>1.2.13</t>
         </is>
       </c>
-      <c r="N87" t="inlineStr"/>
       <c r="O87" t="inlineStr"/>
       <c r="P87" t="inlineStr"/>
       <c r="Q87" s="3" t="n">
@@ -6188,31 +6190,31 @@
           <t>Final Checklist &amp; Upload</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr">
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr">
         <is>
           <t>Media Manager / DIT</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr">
+      <c r="J88" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J88" s="2" t="n">
+      <c r="K88" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K88" s="2" t="n">
+      <c r="L88" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="L88" s="2" t="n">
+      <c r="M88" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M88" t="inlineStr">
+      <c r="N88" t="inlineStr">
         <is>
           <t>1.2.13.1</t>
         </is>
       </c>
-      <c r="N88" t="inlineStr"/>
       <c r="O88" t="inlineStr"/>
       <c r="P88" t="inlineStr"/>
       <c r="Q88" s="3" t="n">
@@ -6256,21 +6258,21 @@
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr"/>
-      <c r="J89" s="2" t="n">
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="K89" s="2" t="n">
+      <c r="L89" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="L89" s="2" t="n">
+      <c r="M89" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="M89" t="inlineStr">
+      <c r="N89" t="inlineStr">
         <is>
           <t>1.2.13</t>
         </is>
       </c>
-      <c r="N89" t="inlineStr"/>
       <c r="O89" t="inlineStr"/>
       <c r="P89" t="inlineStr"/>
       <c r="Q89" s="3" t="n">
@@ -6316,31 +6318,31 @@
           <t>Change Orders &amp; Tracking</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr">
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
         <is>
           <t>Project Manager</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr">
+      <c r="J90" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J90" s="2" t="n">
+      <c r="K90" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K90" s="2" t="n">
+      <c r="L90" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="L90" s="2" t="n">
+      <c r="M90" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M90" t="inlineStr">
+      <c r="N90" t="inlineStr">
         <is>
           <t>1.2.14</t>
         </is>
       </c>
-      <c r="N90" t="inlineStr"/>
       <c r="O90" t="inlineStr"/>
       <c r="P90" t="inlineStr"/>
       <c r="Q90" s="3" t="n">
@@ -6386,31 +6388,31 @@
           <t>Internal Review &amp; Critique</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr">
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr">
         <is>
           <t>Producer</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr">
+      <c r="J91" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J91" s="2" t="n">
+      <c r="K91" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K91" s="2" t="n">
+      <c r="L91" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="L91" s="2" t="n">
+      <c r="M91" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M91" t="inlineStr">
+      <c r="N91" t="inlineStr">
         <is>
           <t>1.2.14.1</t>
         </is>
       </c>
-      <c r="N91" t="inlineStr"/>
       <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr"/>
       <c r="Q91" s="3" t="n">
@@ -6456,31 +6458,31 @@
           <t>Client Review &amp; Revisions</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr">
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr">
         <is>
           <t>Account Manager</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr">
+      <c r="J92" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J92" s="2" t="n">
+      <c r="K92" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K92" s="2" t="n">
+      <c r="L92" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="L92" s="2" t="n">
+      <c r="M92" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M92" t="inlineStr">
+      <c r="N92" t="inlineStr">
         <is>
           <t>1.2.14.2</t>
         </is>
       </c>
-      <c r="N92" t="inlineStr"/>
       <c r="O92" t="inlineStr"/>
       <c r="P92" t="inlineStr"/>
       <c r="Q92" s="3" t="n">
@@ -6526,31 +6528,31 @@
           <t>Invoice Reconciliation</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr">
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr">
         <is>
           <t>Designer</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr">
+      <c r="J93" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J93" s="2" t="n">
+      <c r="K93" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="K93" s="2" t="n">
+      <c r="L93" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="L93" s="2" t="n">
+      <c r="M93" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M93" t="inlineStr">
+      <c r="N93" t="inlineStr">
         <is>
           <t>1.2.14.3</t>
         </is>
       </c>
-      <c r="N93" t="inlineStr"/>
       <c r="O93" t="inlineStr"/>
       <c r="P93" t="inlineStr"/>
       <c r="Q93" s="3" t="n">
@@ -6594,21 +6596,21 @@
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr"/>
       <c r="I94" t="inlineStr"/>
-      <c r="J94" s="2" t="n">
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="K94" s="2" t="n">
+      <c r="L94" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="L94" s="2" t="n">
+      <c r="M94" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="M94" t="inlineStr">
+      <c r="N94" t="inlineStr">
         <is>
           <t>1.2.14</t>
         </is>
       </c>
-      <c r="N94" t="inlineStr"/>
       <c r="O94" t="inlineStr"/>
       <c r="P94" t="inlineStr"/>
       <c r="Q94" s="3" t="n">
@@ -6654,31 +6656,31 @@
           <t>Internal Review &amp; Critique</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr">
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr">
         <is>
           <t>Producer</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr">
+      <c r="J95" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J95" s="2" t="n">
+      <c r="K95" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K95" s="2" t="n">
+      <c r="L95" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="L95" s="2" t="n">
+      <c r="M95" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M95" t="inlineStr">
+      <c r="N95" t="inlineStr">
         <is>
           <t>1.2.15</t>
         </is>
       </c>
-      <c r="N95" t="inlineStr"/>
       <c r="O95" t="inlineStr"/>
       <c r="P95" t="inlineStr"/>
       <c r="Q95" s="3" t="n">
@@ -6724,31 +6726,31 @@
           <t>Client Review &amp; Revisions</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr">
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr">
         <is>
           <t>Account Manager</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr">
+      <c r="J96" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J96" s="2" t="n">
+      <c r="K96" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K96" s="2" t="n">
+      <c r="L96" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="L96" s="2" t="n">
+      <c r="M96" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M96" t="inlineStr">
+      <c r="N96" t="inlineStr">
         <is>
           <t>1.2.15.1</t>
         </is>
       </c>
-      <c r="N96" t="inlineStr"/>
       <c r="O96" t="inlineStr"/>
       <c r="P96" t="inlineStr"/>
       <c r="Q96" s="3" t="n">
@@ -6794,31 +6796,31 @@
           <t>Cutdowns (2-3)</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr">
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr">
         <is>
           <t>Editor</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr">
+      <c r="J97" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J97" s="2" t="n">
+      <c r="K97" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="K97" s="2" t="n">
+      <c r="L97" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="L97" s="2" t="n">
+      <c r="M97" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M97" t="inlineStr">
+      <c r="N97" t="inlineStr">
         <is>
           <t>1.2.15.2</t>
         </is>
       </c>
-      <c r="N97" t="inlineStr"/>
       <c r="O97" t="inlineStr"/>
       <c r="P97" t="inlineStr"/>
       <c r="Q97" s="3" t="n">
@@ -6862,21 +6864,21 @@
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr"/>
       <c r="I98" t="inlineStr"/>
-      <c r="J98" s="2" t="n">
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K98" s="2" t="n">
+      <c r="L98" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="L98" s="2" t="n">
+      <c r="M98" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M98" t="inlineStr">
+      <c r="N98" t="inlineStr">
         <is>
           <t>1.2.15</t>
         </is>
       </c>
-      <c r="N98" t="inlineStr"/>
       <c r="O98" t="inlineStr"/>
       <c r="P98" t="inlineStr"/>
       <c r="Q98" s="3" t="n">
@@ -6922,31 +6924,31 @@
           <t>Client Review Coordination</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr">
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr">
         <is>
           <t>Account Manager</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr">
+      <c r="J99" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J99" s="2" t="n">
+      <c r="K99" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K99" s="2" t="n">
+      <c r="L99" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="L99" s="2" t="n">
+      <c r="M99" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M99" t="inlineStr">
+      <c r="N99" t="inlineStr">
         <is>
           <t>1.2.16</t>
         </is>
       </c>
-      <c r="N99" t="inlineStr"/>
       <c r="O99" t="inlineStr"/>
       <c r="P99" t="inlineStr"/>
       <c r="Q99" s="3" t="n">
@@ -6990,21 +6992,21 @@
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr"/>
       <c r="I100" t="inlineStr"/>
-      <c r="J100" s="2" t="n">
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K100" s="2" t="n">
+      <c r="L100" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="L100" s="2" t="n">
+      <c r="M100" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="M100" t="inlineStr">
+      <c r="N100" t="inlineStr">
         <is>
           <t>1.2.16</t>
         </is>
       </c>
-      <c r="N100" t="inlineStr"/>
       <c r="O100" t="inlineStr"/>
       <c r="P100" t="inlineStr"/>
       <c r="Q100" s="3" t="n">
@@ -7050,31 +7052,31 @@
           <t>Client Review Coordination</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr">
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr">
         <is>
           <t>Account Manager</t>
         </is>
       </c>
-      <c r="I101" t="inlineStr">
+      <c r="J101" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J101" s="2" t="n">
+      <c r="K101" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K101" s="2" t="n">
+      <c r="L101" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="L101" s="2" t="n">
+      <c r="M101" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M101" t="inlineStr">
+      <c r="N101" t="inlineStr">
         <is>
           <t>1.2.17</t>
         </is>
       </c>
-      <c r="N101" t="inlineStr"/>
       <c r="O101" t="inlineStr"/>
       <c r="P101" t="inlineStr"/>
       <c r="Q101" s="3" t="n">
@@ -7120,31 +7122,31 @@
           <t>Notes Triage</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr">
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr">
         <is>
           <t>Project Manager</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr">
+      <c r="J102" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J102" s="2" t="n">
+      <c r="K102" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K102" s="2" t="n">
+      <c r="L102" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="L102" s="2" t="n">
+      <c r="M102" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M102" t="inlineStr">
+      <c r="N102" t="inlineStr">
         <is>
           <t>1.2.17.1</t>
         </is>
       </c>
-      <c r="N102" t="inlineStr"/>
       <c r="O102" t="inlineStr"/>
       <c r="P102" t="inlineStr"/>
       <c r="Q102" s="3" t="n">
@@ -7188,21 +7190,21 @@
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr"/>
       <c r="I103" t="inlineStr"/>
-      <c r="J103" s="2" t="n">
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K103" s="2" t="n">
+      <c r="L103" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="L103" s="2" t="n">
+      <c r="M103" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M103" t="inlineStr">
+      <c r="N103" t="inlineStr">
         <is>
           <t>1.2.17</t>
         </is>
       </c>
-      <c r="N103" t="inlineStr"/>
       <c r="O103" t="inlineStr"/>
       <c r="P103" t="inlineStr"/>
       <c r="Q103" s="3" t="n">
@@ -7248,31 +7250,31 @@
           <t>Post Support</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr">
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr">
         <is>
           <t>Editor</t>
         </is>
       </c>
-      <c r="I104" t="inlineStr">
+      <c r="J104" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J104" s="2" t="n">
+      <c r="K104" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K104" s="2" t="n">
+      <c r="L104" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="L104" s="2" t="n">
+      <c r="M104" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M104" t="inlineStr">
+      <c r="N104" t="inlineStr">
         <is>
           <t>1.2.18</t>
         </is>
       </c>
-      <c r="N104" t="inlineStr"/>
       <c r="O104" t="inlineStr"/>
       <c r="P104" t="inlineStr"/>
       <c r="Q104" s="3" t="n">
@@ -7316,21 +7318,21 @@
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr"/>
-      <c r="J105" s="2" t="n">
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K105" s="2" t="n">
+      <c r="L105" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="L105" s="2" t="n">
+      <c r="M105" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M105" t="inlineStr">
+      <c r="N105" t="inlineStr">
         <is>
           <t>1.2.18</t>
         </is>
       </c>
-      <c r="N105" t="inlineStr"/>
       <c r="O105" t="inlineStr"/>
       <c r="P105" t="inlineStr"/>
       <c r="Q105" s="3" t="n">
@@ -7376,31 +7378,31 @@
           <t>Post Support</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr">
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr">
         <is>
           <t>Editor</t>
         </is>
       </c>
-      <c r="I106" t="inlineStr">
+      <c r="J106" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J106" s="2" t="n">
+      <c r="K106" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K106" s="2" t="n">
+      <c r="L106" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="L106" s="2" t="n">
+      <c r="M106" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M106" t="inlineStr">
+      <c r="N106" t="inlineStr">
         <is>
           <t>1.2.19</t>
         </is>
       </c>
-      <c r="N106" t="inlineStr"/>
       <c r="O106" t="inlineStr"/>
       <c r="P106" t="inlineStr"/>
       <c r="Q106" s="3" t="n">
@@ -7444,21 +7446,21 @@
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr"/>
       <c r="I107" t="inlineStr"/>
-      <c r="J107" s="2" t="n">
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K107" s="2" t="n">
+      <c r="L107" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="L107" s="2" t="n">
+      <c r="M107" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M107" t="inlineStr">
+      <c r="N107" t="inlineStr">
         <is>
           <t>1.2.19</t>
         </is>
       </c>
-      <c r="N107" t="inlineStr"/>
       <c r="O107" t="inlineStr"/>
       <c r="P107" t="inlineStr"/>
       <c r="Q107" s="3" t="n">
@@ -7504,31 +7506,31 @@
           <t>Post Support</t>
         </is>
       </c>
-      <c r="H108" t="inlineStr">
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr">
         <is>
           <t>Editor</t>
         </is>
       </c>
-      <c r="I108" t="inlineStr">
+      <c r="J108" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J108" s="2" t="n">
+      <c r="K108" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K108" s="2" t="n">
+      <c r="L108" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="L108" s="2" t="n">
+      <c r="M108" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M108" t="inlineStr">
+      <c r="N108" t="inlineStr">
         <is>
           <t>1.2.20</t>
         </is>
       </c>
-      <c r="N108" t="inlineStr"/>
       <c r="O108" t="inlineStr"/>
       <c r="P108" t="inlineStr"/>
       <c r="Q108" s="3" t="n">
@@ -7572,21 +7574,21 @@
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr"/>
-      <c r="J109" s="2" t="n">
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="K109" s="2" t="n">
+      <c r="L109" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="L109" s="2" t="n">
+      <c r="M109" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M109" t="inlineStr">
+      <c r="N109" t="inlineStr">
         <is>
           <t>1.2.20</t>
         </is>
       </c>
-      <c r="N109" t="inlineStr"/>
       <c r="O109" t="inlineStr"/>
       <c r="P109" t="inlineStr"/>
       <c r="Q109" s="3" t="n">
@@ -7632,31 +7634,31 @@
           <t>Post Support</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr">
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr">
         <is>
           <t>Editor</t>
         </is>
       </c>
-      <c r="I110" t="inlineStr">
+      <c r="J110" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J110" s="2" t="n">
+      <c r="K110" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="K110" s="2" t="n">
+      <c r="L110" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="L110" s="2" t="n">
+      <c r="M110" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M110" t="inlineStr">
+      <c r="N110" t="inlineStr">
         <is>
           <t>1.2.21</t>
         </is>
       </c>
-      <c r="N110" t="inlineStr"/>
       <c r="O110" t="inlineStr"/>
       <c r="P110" t="inlineStr"/>
       <c r="Q110" s="3" t="n">
@@ -7700,21 +7702,21 @@
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr"/>
-      <c r="J111" s="2" t="n">
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="K111" s="2" t="n">
+      <c r="L111" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="L111" s="2" t="n">
+      <c r="M111" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M111" t="inlineStr">
+      <c r="N111" t="inlineStr">
         <is>
           <t>1.2.21</t>
         </is>
       </c>
-      <c r="N111" t="inlineStr"/>
       <c r="O111" t="inlineStr"/>
       <c r="P111" t="inlineStr"/>
       <c r="Q111" s="3" t="n">
@@ -7760,31 +7762,31 @@
           <t>Post Support</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr">
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr">
         <is>
           <t>Editor</t>
         </is>
       </c>
-      <c r="I112" t="inlineStr">
+      <c r="J112" t="inlineStr">
         <is>
           <t>Mid</t>
         </is>
       </c>
-      <c r="J112" s="2" t="n">
+      <c r="K112" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="K112" s="2" t="n">
+      <c r="L112" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="L112" s="2" t="n">
+      <c r="M112" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M112" t="inlineStr">
+      <c r="N112" t="inlineStr">
         <is>
           <t>1.2.22</t>
         </is>
       </c>
-      <c r="N112" t="inlineStr"/>
       <c r="O112" t="inlineStr"/>
       <c r="P112" t="inlineStr"/>
       <c r="Q112" s="3" t="n">

</xml_diff>